<commit_message>
Completed Till Week 10
</commit_message>
<xml_diff>
--- a/Docs/Nisharg Soni-G2.xlsx
+++ b/Docs/Nisharg Soni-G2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\NishargSoni-458\RKIT_TRAINING\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DE98DB9-3557-45E1-8EEB-F5A6FE752EFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19990A69-7DE3-447B-B5B3-9D4A0FC4DE6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="836" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="836" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="12" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="Version Control (Git)" sheetId="11" r:id="rId8"/>
     <sheet name="Architecture + Coding" sheetId="14" r:id="rId9"/>
     <sheet name="Other" sheetId="15" r:id="rId10"/>
+    <sheet name="Sheet1" sheetId="16" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -1766,6 +1767,15 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C444A79-06FC-4DA0-9E55-0CFA536F9164}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B59A8890-A43A-49B0-868B-EB9D50B09E63}">
   <dimension ref="A1:K13"/>
@@ -3603,7 +3613,7 @@
         <v>46007</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>238</v>
@@ -3632,7 +3642,7 @@
         <v>46008</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>238</v>
@@ -3661,7 +3671,7 @@
         <v>46010</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>238</v>
@@ -3690,7 +3700,7 @@
         <v>46010</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>238</v>
@@ -3719,7 +3729,7 @@
         <v>46011</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>238</v>
@@ -3748,7 +3758,7 @@
         <v>46013</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>238</v>
@@ -3777,7 +3787,7 @@
         <v>46013</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>238</v>
@@ -3803,7 +3813,7 @@
         <v>46014</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>238</v>
@@ -3829,7 +3839,7 @@
         <v>46016</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>238</v>
@@ -3855,7 +3865,7 @@
         <v>46016</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>238</v>
@@ -3881,7 +3891,7 @@
         <v>46017</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>238</v>
@@ -4086,7 +4096,7 @@
         <v>236</v>
       </c>
       <c r="G7" s="11">
-        <v>46030</v>
+        <v>46031</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -4494,18 +4504,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4647,18 +4657,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55EF8721-4A61-4D2C-A16B-F3152A60B6FA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56DCEFB2-4877-4926-B462-8A1B0C5C05F8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56DCEFB2-4877-4926-B462-8A1B0C5C05F8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55EF8721-4A61-4D2C-A16B-F3152A60B6FA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update Nisharg Soni-G2.xlsx with new changes
</commit_message>
<xml_diff>
--- a/Docs/Nisharg Soni-G2.xlsx
+++ b/Docs/Nisharg Soni-G2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\NishargSoni-458\RKIT_TRAINING\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19990A69-7DE3-447B-B5B3-9D4A0FC4DE6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA48D171-1FAF-41B9-A4DA-1A2A96D5FE67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="836" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="836" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="12" r:id="rId1"/>
@@ -2879,7 +2879,7 @@
         <v>237</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -2908,7 +2908,7 @@
         <v>237</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -2937,7 +2937,7 @@
         <v>237</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -2966,7 +2966,7 @@
         <v>237</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -2995,7 +2995,7 @@
         <v>237</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -3024,7 +3024,7 @@
         <v>237</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -3053,7 +3053,7 @@
         <v>237</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -3082,7 +3082,7 @@
         <v>237</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -3111,7 +3111,7 @@
         <v>237</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -3140,7 +3140,7 @@
         <v>237</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -3169,7 +3169,7 @@
         <v>237</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -3198,7 +3198,7 @@
         <v>237</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -3291,7 +3291,7 @@
         <v>237</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -3320,7 +3320,7 @@
         <v>237</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -3349,7 +3349,7 @@
         <v>237</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -3378,7 +3378,7 @@
         <v>237</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -3407,7 +3407,7 @@
         <v>237</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -3436,7 +3436,7 @@
         <v>237</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -3465,7 +3465,7 @@
         <v>237</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -3494,7 +3494,7 @@
         <v>237</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -3523,7 +3523,7 @@
         <v>237</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -4073,7 +4073,7 @@
         <v>236</v>
       </c>
       <c r="G6" s="11">
-        <v>46030</v>
+        <v>46031</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -4096,7 +4096,7 @@
         <v>236</v>
       </c>
       <c r="G7" s="11">
-        <v>46031</v>
+        <v>46034</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -4510,15 +4510,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F3C32926E4737E47B27DDAA5D371959A" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="10250be6089a57ac4e60aefa3d8c7247">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a7998c3e-7f65-4586-b9f5-db7168bdbc10" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f71cd174da29f72f20168de9339b0a7a" ns2:_="">
     <xsd:import namespace="a7998c3e-7f65-4586-b9f5-db7168bdbc10"/>
@@ -4656,6 +4647,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56DCEFB2-4877-4926-B462-8A1B0C5C05F8}">
   <ds:schemaRefs>
@@ -4666,14 +4666,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55EF8721-4A61-4D2C-A16B-F3152A60B6FA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA151C35-975C-4B59-AE26-DA6BD662A7F0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4689,4 +4681,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55EF8721-4A61-4D2C-A16B-F3152A60B6FA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added Week 10 Notes
</commit_message>
<xml_diff>
--- a/Docs/Nisharg Soni-G2.xlsx
+++ b/Docs/Nisharg Soni-G2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\NishargSoni-458\RKIT_TRAINING\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA48D171-1FAF-41B9-A4DA-1A2A96D5FE67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF4D1D99-E3B9-4497-80DD-30F85B625EFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="836" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4510,6 +4510,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F3C32926E4737E47B27DDAA5D371959A" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="10250be6089a57ac4e60aefa3d8c7247">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a7998c3e-7f65-4586-b9f5-db7168bdbc10" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f71cd174da29f72f20168de9339b0a7a" ns2:_="">
     <xsd:import namespace="a7998c3e-7f65-4586-b9f5-db7168bdbc10"/>
@@ -4647,15 +4656,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56DCEFB2-4877-4926-B462-8A1B0C5C05F8}">
   <ds:schemaRefs>
@@ -4666,6 +4666,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55EF8721-4A61-4D2C-A16B-F3152A60B6FA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA151C35-975C-4B59-AE26-DA6BD662A7F0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4681,12 +4689,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55EF8721-4A61-4D2C-A16B-F3152A60B6FA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added Demos for .net
</commit_message>
<xml_diff>
--- a/Docs/Nisharg Soni-G2.xlsx
+++ b/Docs/Nisharg Soni-G2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\NishargSoni-458\RKIT_TRAINING\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD1A27CC-A427-49EB-B7EB-FF834D448FAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8557104-298B-43DF-833B-0DAE1D358172}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2940" windowWidth="15375" windowHeight="7875" tabRatio="836" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="836" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="12" r:id="rId1"/>
@@ -4510,15 +4510,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F3C32926E4737E47B27DDAA5D371959A" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="10250be6089a57ac4e60aefa3d8c7247">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a7998c3e-7f65-4586-b9f5-db7168bdbc10" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f71cd174da29f72f20168de9339b0a7a" ns2:_="">
     <xsd:import namespace="a7998c3e-7f65-4586-b9f5-db7168bdbc10"/>
@@ -4656,6 +4647,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56DCEFB2-4877-4926-B462-8A1B0C5C05F8}">
   <ds:schemaRefs>
@@ -4666,14 +4666,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55EF8721-4A61-4D2C-A16B-F3152A60B6FA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA151C35-975C-4B59-AE26-DA6BD662A7F0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4689,4 +4681,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55EF8721-4A61-4D2C-A16B-F3152A60B6FA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>